<commit_message>
curation: record unmatched variants, drop the inactive priority draw, document benchmark provenance (closes #3, #4)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curation_benchmark/results/supp_tables/supp_table_dataset_counts.xlsx
+++ b/curation_benchmark/results/supp_tables/supp_table_dataset_counts.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dataset_counts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dbnsfp_match" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1580,4 +1581,596 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>coordinate_list</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_in_list</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>n_in_database</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>match_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MSK_hotspot</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>hg38</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hotspot_annotation_fordb_withouttranscript_gd.txt</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1020</v>
+      </c>
+      <c r="E2" t="n">
+        <v>826</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.8098</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MSK_passenger</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MSK_passenger_hg19_annotation_6246.txt</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6239</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6234</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9992</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TCGA_passenger</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TCGA_passenger_hg19_annotation_rd5000.txt</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Alpha_pos</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hg38</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>alphamissense_cancer_pos.txt</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>868</v>
+      </c>
+      <c r="E5" t="n">
+        <v>862</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9931</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alpha_neg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hg38</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>alphamissense_cancer_neg.txt</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1733</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1733</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ASD_case1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hg38</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ASD_study1_case_hg38_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1331</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1312</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9857</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ASD_case2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ASD_study2_case_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2783</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2728</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.9802</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ASD_case3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ASD_study3_case_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1653</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1631</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.9867</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ASD_case4</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ASD_study4_case_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>125</v>
+      </c>
+      <c r="E10" t="n">
+        <v>105</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ASD_pri_case1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ASD_primate_study1.txt</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1107</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1094</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.9883</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ASD_pri_case2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ASD_primate_study2_case.txt</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>207</v>
+      </c>
+      <c r="E12" t="n">
+        <v>203</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.9807</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ASD_pri_case3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ASD_primate_study3.txt</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>143</v>
+      </c>
+      <c r="E13" t="n">
+        <v>141</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.986</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CHD_case</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CHD_case_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1924</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1905</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.9901</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DDD_case</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DDD_case_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3787</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3643</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.962</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DDD_pri_case1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DDD_primate_study1.txt</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>862</v>
+      </c>
+      <c r="E16" t="n">
+        <v>832</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.9651999999999999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DDD_pri_case2</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>DDD_primate_study2.txt</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>28240</v>
+      </c>
+      <c r="E17" t="n">
+        <v>26666</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.9443</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>control1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>hg38</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ASD_study1_control_hg38_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1219</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1196</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.9811</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>control2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ASD_study2_control_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1347</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1306</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.9696</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>control3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ASD_study3_control_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1128</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1112</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.9858</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>control4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ASD_study4_control_hg19_annotation.txt</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>82</v>
+      </c>
+      <c r="E21" t="n">
+        <v>65</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.7927</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pri_control2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>hg19</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ASD_primate_study2_control.txt</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>207</v>
+      </c>
+      <c r="E22" t="n">
+        <v>198</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.9565</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
curation: resolve IUPAC ambiguity codes and complete the study-4 filters
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curation_benchmark/results/supp_tables/supp_table_dataset_counts.xlsx
+++ b/curation_benchmark/results/supp_tables/supp_table_dataset_counts.xlsx
@@ -1852,10 +1852,10 @@
         <v>125</v>
       </c>
       <c r="E10" t="n">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="F10" t="n">
-        <v>0.84</v>
+        <v>0.992</v>
       </c>
     </row>
     <row r="11">
@@ -2138,10 +2138,10 @@
         <v>82</v>
       </c>
       <c r="E21" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7927</v>
+        <v>0.9756</v>
       </c>
     </row>
     <row r="22">

</xml_diff>